<commit_message>
feat: 補上 rogue-1/rogue-2/orc/wolf/horse 的顯示名稱（含英文）
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/xls/local.xlsx
+++ b/xls/local.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="586" uniqueCount="497">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="596" uniqueCount="505">
   <si>
     <t>key</t>
   </si>
@@ -667,6 +667,30 @@
   </si>
   <si>
     <t>guard-2</t>
+  </si>
+  <si>
+    <t>rogue-1</t>
+  </si>
+  <si>
+    <t>rogue-2</t>
+  </si>
+  <si>
+    <t>orc</t>
+  </si>
+  <si>
+    <t>獸人</t>
+  </si>
+  <si>
+    <t>wolf</t>
+  </si>
+  <si>
+    <t>狼</t>
+  </si>
+  <si>
+    <t>horse</t>
+  </si>
+  <si>
+    <t>馬</t>
   </si>
   <si>
     <t>ranger</t>
@@ -2869,40 +2893,40 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>394</v>
+        <v>402</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>395</v>
+        <v>403</v>
       </c>
       <c r="D15" s="3"/>
       <c r="E15" s="3"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>396</v>
+        <v>404</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>397</v>
+        <v>405</v>
       </c>
       <c r="D16" s="3"/>
       <c r="E16" s="3"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>398</v>
+        <v>406</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>399</v>
+        <v>407</v>
       </c>
       <c r="D17" s="3"/>
       <c r="E17" s="3"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>226</v>
+        <v>234</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>400</v>
+        <v>408</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" s="3"/>
@@ -2910,10 +2934,10 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>401</v>
+        <v>409</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>402</v>
+        <v>410</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" s="3"/>
@@ -2960,421 +2984,421 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>403</v>
+        <v>411</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>404</v>
+        <v>412</v>
       </c>
       <c r="C3" s="2"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>405</v>
+        <v>413</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>406</v>
+        <v>414</v>
       </c>
       <c r="C4" s="2"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>407</v>
+        <v>415</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>408</v>
+        <v>416</v>
       </c>
       <c r="C5" s="2"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>410</v>
+        <v>418</v>
       </c>
       <c r="C6" s="2"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>411</v>
+        <v>419</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="C7" s="2"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>413</v>
+        <v>421</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>414</v>
+        <v>422</v>
       </c>
       <c r="C8" s="2"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>415</v>
+        <v>423</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>416</v>
+        <v>424</v>
       </c>
       <c r="C9" s="2"/>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>417</v>
+        <v>425</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>418</v>
+        <v>426</v>
       </c>
       <c r="C10" s="2"/>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>419</v>
+        <v>427</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>420</v>
+        <v>428</v>
       </c>
       <c r="C11" s="2"/>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>421</v>
+        <v>429</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>422</v>
+        <v>430</v>
       </c>
       <c r="C12" s="2"/>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>423</v>
+        <v>431</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>424</v>
+        <v>432</v>
       </c>
       <c r="C13" s="2"/>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>425</v>
+        <v>433</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>426</v>
+        <v>434</v>
       </c>
       <c r="C14" s="2"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>427</v>
+        <v>435</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>428</v>
+        <v>436</v>
       </c>
       <c r="C15" s="2"/>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>429</v>
+        <v>437</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>430</v>
+        <v>438</v>
       </c>
       <c r="C16" s="2"/>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>431</v>
+        <v>439</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>432</v>
+        <v>440</v>
       </c>
       <c r="C17" s="2"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>433</v>
+        <v>441</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>434</v>
+        <v>442</v>
       </c>
       <c r="C18" s="2"/>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>435</v>
+        <v>443</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>436</v>
+        <v>444</v>
       </c>
       <c r="C19" s="2"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>437</v>
+        <v>445</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>438</v>
+        <v>446</v>
       </c>
       <c r="C20" s="2"/>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>439</v>
+        <v>447</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>440</v>
+        <v>448</v>
       </c>
       <c r="C21" s="2"/>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>441</v>
+        <v>449</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>442</v>
+        <v>450</v>
       </c>
       <c r="C22" s="2"/>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>443</v>
+        <v>451</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>444</v>
+        <v>452</v>
       </c>
       <c r="C23" s="2"/>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>445</v>
+        <v>453</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>446</v>
+        <v>454</v>
       </c>
       <c r="C24" s="2"/>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>447</v>
+        <v>455</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>448</v>
+        <v>456</v>
       </c>
       <c r="C25" s="2"/>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>449</v>
+        <v>457</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>450</v>
+        <v>458</v>
       </c>
       <c r="C26" s="2"/>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>451</v>
+        <v>459</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>452</v>
+        <v>460</v>
       </c>
       <c r="C27" s="2"/>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>453</v>
+        <v>461</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>454</v>
+        <v>462</v>
       </c>
       <c r="C28" s="2"/>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>455</v>
+        <v>463</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>456</v>
+        <v>464</v>
       </c>
       <c r="C29" s="2"/>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>457</v>
+        <v>465</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>458</v>
+        <v>466</v>
       </c>
       <c r="C30" s="2"/>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>459</v>
+        <v>467</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>460</v>
+        <v>468</v>
       </c>
       <c r="C31" s="2"/>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>461</v>
+        <v>469</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>462</v>
+        <v>470</v>
       </c>
       <c r="C32" s="2"/>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>463</v>
+        <v>471</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>464</v>
+        <v>472</v>
       </c>
       <c r="C33" s="2"/>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>465</v>
+        <v>473</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>466</v>
+        <v>474</v>
       </c>
       <c r="C34" s="2"/>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>467</v>
+        <v>475</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>468</v>
+        <v>476</v>
       </c>
       <c r="C35" s="2"/>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>469</v>
+        <v>477</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>470</v>
+        <v>478</v>
       </c>
       <c r="C36" s="2"/>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>471</v>
+        <v>479</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>472</v>
+        <v>480</v>
       </c>
       <c r="C37" s="2"/>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>473</v>
+        <v>481</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>474</v>
+        <v>482</v>
       </c>
       <c r="C38" s="2"/>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>475</v>
+        <v>483</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>476</v>
+        <v>484</v>
       </c>
       <c r="C39" s="2"/>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>477</v>
+        <v>485</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>478</v>
+        <v>486</v>
       </c>
       <c r="C40" s="2"/>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>479</v>
+        <v>487</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>480</v>
+        <v>488</v>
       </c>
       <c r="C41" s="2"/>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>481</v>
+        <v>489</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>482</v>
+        <v>490</v>
       </c>
       <c r="C42" s="2"/>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>483</v>
+        <v>491</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>484</v>
+        <v>492</v>
       </c>
       <c r="C43" s="2"/>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>485</v>
+        <v>493</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>486</v>
+        <v>494</v>
       </c>
       <c r="C44" s="2"/>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
-        <v>487</v>
+        <v>495</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>488</v>
+        <v>496</v>
       </c>
       <c r="C45" s="2"/>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>489</v>
+        <v>497</v>
       </c>
       <c r="B46" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>491</v>
+        <v>499</v>
       </c>
       <c r="B47" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>493</v>
+        <v>501</v>
       </c>
       <c r="B48" t="s">
-        <v>494</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>495</v>
+        <v>503</v>
       </c>
       <c r="B49" t="s">
-        <v>496</v>
+        <v>504</v>
       </c>
     </row>
   </sheetData>
@@ -3846,23 +3870,53 @@
       <c r="E14" s="6"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="7"/>
+      <c r="A15" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="C15" s="9"/>
       <c r="D15" s="8"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="7"/>
+      <c r="A16" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="C16" s="9"/>
       <c r="D16" s="8"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="7"/>
+      <c r="A17" s="7" t="s">
+        <v>216</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>217</v>
+      </c>
+      <c r="C17" s="9"/>
       <c r="D17" s="8"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="7"/>
+      <c r="A18" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="C18" s="9"/>
       <c r="D18" s="8"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="7"/>
+      <c r="A19" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="C19" s="9"/>
       <c r="D19" s="8"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -3955,13 +4009,13 @@
     </row>
     <row r="3" ht="31.5" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
@@ -3971,78 +4025,78 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
-        <v>217</v>
+        <v>225</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="D5" s="13"/>
       <c r="E5" s="3"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>220</v>
+        <v>228</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="D6" s="13"/>
       <c r="E6" s="3"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="D7" s="13"/>
       <c r="E7" s="3"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>226</v>
+        <v>234</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>228</v>
+        <v>236</v>
       </c>
       <c r="D8" s="13"/>
       <c r="E8" s="3"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>230</v>
+        <v>238</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>231</v>
+        <v>239</v>
       </c>
       <c r="D9" s="13"/>
       <c r="E9" s="3"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
-        <v>232</v>
+        <v>240</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>211</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="D10" s="13"/>
       <c r="E10" s="3"/>
@@ -4173,65 +4227,65 @@
     </row>
     <row r="3" ht="16.5" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>234</v>
+        <v>242</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>235</v>
+        <v>243</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>236</v>
+        <v>244</v>
       </c>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>238</v>
+        <v>246</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>239</v>
+        <v>247</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>240</v>
+        <v>248</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>241</v>
+        <v>249</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>242</v>
+        <v>250</v>
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="3"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>243</v>
+        <v>251</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>246</v>
+        <v>254</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
@@ -4242,10 +4296,10 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>250</v>
+        <v>258</v>
       </c>
       <c r="C9" s="18"/>
       <c r="D9" s="3"/>
@@ -4253,104 +4307,104 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="B10" s="18" t="s">
         <v>51</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>252</v>
+        <v>260</v>
       </c>
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>253</v>
+        <v>261</v>
       </c>
       <c r="B11" s="18" t="s">
         <v>54</v>
       </c>
       <c r="C11" s="18" t="s">
-        <v>254</v>
+        <v>262</v>
       </c>
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>255</v>
+        <v>263</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>256</v>
+        <v>264</v>
       </c>
       <c r="C12" s="18" t="s">
-        <v>257</v>
+        <v>265</v>
       </c>
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>258</v>
+        <v>266</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="C13" s="18" t="s">
-        <v>260</v>
+        <v>268</v>
       </c>
       <c r="D13" s="3"/>
       <c r="E13" s="3"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>262</v>
+        <v>270</v>
       </c>
       <c r="C14" s="18" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="D14" s="3"/>
       <c r="E14" s="3"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>264</v>
+        <v>272</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>265</v>
+        <v>273</v>
       </c>
       <c r="C15" s="18" t="s">
-        <v>266</v>
+        <v>274</v>
       </c>
       <c r="D15" s="3"/>
       <c r="E15" s="3"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>267</v>
+        <v>275</v>
       </c>
       <c r="B16" s="18" t="s">
-        <v>268</v>
+        <v>276</v>
       </c>
       <c r="C16" s="18" t="s">
-        <v>269</v>
+        <v>277</v>
       </c>
       <c r="D16" s="3"/>
       <c r="E16" s="3"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>270</v>
+        <v>278</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>271</v>
+        <v>279</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>272</v>
+        <v>280</v>
       </c>
       <c r="D17" s="3"/>
       <c r="E17" s="3"/>
@@ -4361,10 +4415,10 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>273</v>
+        <v>281</v>
       </c>
       <c r="B19" s="18" t="s">
-        <v>274</v>
+        <v>282</v>
       </c>
       <c r="C19" s="18"/>
       <c r="D19" s="3"/>
@@ -4372,52 +4426,52 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>275</v>
+        <v>283</v>
       </c>
       <c r="B20" s="18" t="s">
-        <v>276</v>
+        <v>284</v>
       </c>
       <c r="C20" s="18" t="s">
-        <v>277</v>
+        <v>285</v>
       </c>
       <c r="D20" s="3"/>
       <c r="E20" s="3"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>278</v>
+        <v>286</v>
       </c>
       <c r="B21" s="18" t="s">
-        <v>279</v>
+        <v>287</v>
       </c>
       <c r="C21" s="18" t="s">
-        <v>280</v>
+        <v>288</v>
       </c>
       <c r="D21" s="3"/>
       <c r="E21" s="3"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>281</v>
+        <v>289</v>
       </c>
       <c r="B22" s="18" t="s">
-        <v>282</v>
+        <v>290</v>
       </c>
       <c r="C22" s="18" t="s">
-        <v>283</v>
+        <v>291</v>
       </c>
       <c r="D22" s="3"/>
       <c r="E22" s="3"/>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>284</v>
+        <v>292</v>
       </c>
       <c r="B23" s="18" t="s">
-        <v>285</v>
+        <v>293</v>
       </c>
       <c r="C23" s="18" t="s">
-        <v>286</v>
+        <v>294</v>
       </c>
       <c r="D23" s="3"/>
       <c r="E23" s="3"/>
@@ -4428,10 +4482,10 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>287</v>
+        <v>295</v>
       </c>
       <c r="B25" s="18" t="s">
-        <v>288</v>
+        <v>296</v>
       </c>
       <c r="C25" s="18"/>
       <c r="D25" s="3"/>
@@ -4439,10 +4493,10 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>289</v>
+        <v>297</v>
       </c>
       <c r="B26" s="18" t="s">
-        <v>290</v>
+        <v>298</v>
       </c>
       <c r="C26" s="18"/>
       <c r="D26" s="3"/>
@@ -4450,10 +4504,10 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>291</v>
+        <v>299</v>
       </c>
       <c r="B27" s="18" t="s">
-        <v>292</v>
+        <v>300</v>
       </c>
       <c r="C27" s="18"/>
       <c r="D27" s="3"/>
@@ -4461,10 +4515,10 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>293</v>
+        <v>301</v>
       </c>
       <c r="B28" s="18" t="s">
-        <v>294</v>
+        <v>302</v>
       </c>
       <c r="C28" s="18"/>
       <c r="D28" s="3"/>
@@ -4472,10 +4526,10 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>295</v>
+        <v>303</v>
       </c>
       <c r="B29" s="18" t="s">
-        <v>296</v>
+        <v>304</v>
       </c>
       <c r="C29" s="18"/>
       <c r="D29" s="3"/>
@@ -4487,7 +4541,7 @@
     </row>
     <row r="31" ht="31.5" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>297</v>
+        <v>305</v>
       </c>
       <c r="B31" s="18" t="s">
         <v>48</v>
@@ -4500,26 +4554,26 @@
     </row>
     <row r="32" ht="31.5" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>298</v>
+        <v>306</v>
       </c>
       <c r="B32" s="18" t="s">
-        <v>299</v>
+        <v>307</v>
       </c>
       <c r="C32" s="19" t="s">
-        <v>300</v>
+        <v>308</v>
       </c>
       <c r="D32" s="3"/>
       <c r="E32" s="3"/>
     </row>
     <row r="33" ht="31.5" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>301</v>
+        <v>309</v>
       </c>
       <c r="B33" s="18" t="s">
-        <v>302</v>
+        <v>310</v>
       </c>
       <c r="C33" s="19" t="s">
-        <v>303</v>
+        <v>311</v>
       </c>
       <c r="D33" s="3"/>
       <c r="E33" s="3"/>
@@ -4530,138 +4584,138 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>304</v>
+        <v>312</v>
       </c>
       <c r="B35" s="18" t="s">
-        <v>305</v>
+        <v>313</v>
       </c>
       <c r="C35" s="19" t="s">
-        <v>306</v>
+        <v>314</v>
       </c>
       <c r="D35" s="3"/>
       <c r="E35" s="3"/>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="B36" s="18" t="s">
-        <v>308</v>
+        <v>316</v>
       </c>
       <c r="C36" s="19" t="s">
-        <v>309</v>
+        <v>317</v>
       </c>
       <c r="D36" s="3"/>
       <c r="E36" s="3"/>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>310</v>
+        <v>318</v>
       </c>
       <c r="B37" s="18" t="s">
-        <v>311</v>
+        <v>319</v>
       </c>
       <c r="C37" s="19" t="s">
-        <v>312</v>
+        <v>320</v>
       </c>
       <c r="D37" s="3"/>
       <c r="E37" s="3"/>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="B39" s="18" t="s">
         <v>313</v>
       </c>
-      <c r="B39" s="18" t="s">
-        <v>305</v>
-      </c>
       <c r="C39" s="19" t="s">
-        <v>314</v>
+        <v>322</v>
       </c>
       <c r="D39" s="3"/>
       <c r="E39" s="3"/>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>315</v>
+        <v>323</v>
       </c>
       <c r="B40" s="18" t="s">
-        <v>308</v>
+        <v>316</v>
       </c>
       <c r="C40" s="19" t="s">
-        <v>316</v>
+        <v>324</v>
       </c>
       <c r="D40" s="3"/>
       <c r="E40" s="3"/>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>317</v>
+        <v>325</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>311</v>
+        <v>319</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>318</v>
+        <v>326</v>
       </c>
       <c r="D41" s="3"/>
       <c r="E41" s="3"/>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>319</v>
+        <v>327</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>320</v>
+        <v>328</v>
       </c>
       <c r="D43" s="3"/>
       <c r="E43" s="3"/>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>321</v>
+        <v>329</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>322</v>
+        <v>330</v>
       </c>
       <c r="D44" s="3"/>
       <c r="E44" s="3"/>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
-        <v>323</v>
+        <v>331</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="D45" s="3"/>
       <c r="E45" s="3"/>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
-        <v>324</v>
+        <v>332</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="D46" s="3"/>
       <c r="E46" s="3"/>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
-        <v>326</v>
+        <v>334</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>327</v>
+        <v>335</v>
       </c>
       <c r="D48" s="3"/>
       <c r="E48" s="3"/>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
-        <v>328</v>
+        <v>336</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>329</v>
+        <v>337</v>
       </c>
       <c r="C49" s="4"/>
       <c r="D49" s="3"/>
@@ -4669,33 +4723,33 @@
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
-        <v>330</v>
+        <v>338</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>331</v>
+        <v>339</v>
       </c>
       <c r="D51" s="3"/>
       <c r="E51" s="3"/>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
-        <v>332</v>
+        <v>340</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>333</v>
+        <v>341</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="D52" s="3"/>
       <c r="E52" s="3"/>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>336</v>
+        <v>344</v>
       </c>
       <c r="C53" s="4"/>
       <c r="D53" s="3"/>
@@ -4703,40 +4757,40 @@
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
-        <v>337</v>
+        <v>345</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>338</v>
+        <v>346</v>
       </c>
       <c r="D54" s="3"/>
       <c r="E54" s="3"/>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
-        <v>339</v>
+        <v>347</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>340</v>
+        <v>348</v>
       </c>
       <c r="D55" s="3"/>
       <c r="E55" s="3"/>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D56" s="3"/>
       <c r="E56" s="3"/>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>344</v>
+        <v>352</v>
       </c>
       <c r="D57" s="3"/>
       <c r="E57" s="3"/>
@@ -4781,26 +4835,26 @@
     <row r="3" ht="17.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>345</v>
+        <v>353</v>
       </c>
       <c r="B4" t="s">
-        <v>346</v>
+        <v>354</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>347</v>
+        <v>355</v>
       </c>
       <c r="B5" t="s">
-        <v>348</v>
+        <v>356</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>349</v>
+        <v>357</v>
       </c>
       <c r="B6" t="s">
-        <v>350</v>
+        <v>358</v>
       </c>
     </row>
   </sheetData>
@@ -4845,20 +4899,20 @@
     <row r="3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>351</v>
+        <v>359</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>352</v>
+        <v>360</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>353</v>
+        <v>361</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>354</v>
+        <v>362</v>
       </c>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
@@ -4875,33 +4929,33 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>355</v>
+        <v>363</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>338</v>
+        <v>346</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>356</v>
+        <v>364</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>357</v>
+        <v>365</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>358</v>
+        <v>366</v>
       </c>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>359</v>
+        <v>367</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
@@ -4916,10 +4970,10 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>361</v>
+        <v>369</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>362</v>
+        <v>370</v>
       </c>
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
@@ -4927,10 +4981,10 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>363</v>
+        <v>371</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>364</v>
+        <v>372</v>
       </c>
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
@@ -4938,10 +4992,10 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>365</v>
+        <v>373</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>366</v>
+        <v>374</v>
       </c>
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
@@ -4991,50 +5045,50 @@
     <row r="3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>367</v>
+        <v>375</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>368</v>
+        <v>376</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>369</v>
+        <v>377</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>370</v>
+        <v>378</v>
       </c>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>371</v>
+        <v>379</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>372</v>
+        <v>380</v>
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>373</v>
+        <v>381</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>374</v>
+        <v>382</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>375</v>
+        <v>383</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>376</v>
+        <v>384</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -5076,74 +5130,74 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>377</v>
+        <v>385</v>
       </c>
       <c r="B3" t="s">
-        <v>378</v>
+        <v>386</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>379</v>
+        <v>387</v>
       </c>
       <c r="B4" t="s">
-        <v>380</v>
+        <v>388</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>381</v>
+        <v>389</v>
       </c>
       <c r="B5" t="s">
-        <v>382</v>
+        <v>390</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>383</v>
+        <v>391</v>
       </c>
       <c r="B6" t="s">
-        <v>384</v>
+        <v>392</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>385</v>
+        <v>393</v>
       </c>
       <c r="B7" t="s">
-        <v>386</v>
+        <v>394</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>387</v>
+        <v>395</v>
       </c>
       <c r="B8" t="s">
-        <v>388</v>
+        <v>396</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>389</v>
+        <v>397</v>
       </c>
       <c r="B9" t="s">
-        <v>390</v>
+        <v>398</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>391</v>
+        <v>399</v>
       </c>
       <c r="B10" t="s">
-        <v>350</v>
+        <v>358</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>392</v>
+        <v>400</v>
       </c>
       <c r="B12" t="s">
-        <v>393</v>
+        <v>401</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor: 角色 lab/des 從 local.xlsx 搬進 role.json，情境改 role.<id>，Role 加 label/des getter
</commit_message>
<xml_diff>
--- a/xls/local.xlsx
+++ b/xls/local.xlsx
@@ -9,22 +9,21 @@
   <sheets>
     <sheet sheetId="1" name="general" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="items" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="roles" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="jobs" state="visible" r:id="rId7"/>
-    <sheet sheetId="5" name="stat" state="visible" r:id="rId8"/>
-    <sheet sheetId="6" name="tag" state="visible" r:id="rId9"/>
-    <sheet sheetId="7" name="other" state="visible" r:id="rId10"/>
-    <sheet sheetId="8" name="quest" state="visible" r:id="rId11"/>
-    <sheet sheetId="9" name="ability" state="visible" r:id="rId12"/>
-    <sheet sheetId="10" name="option" state="visible" r:id="rId13"/>
-    <sheet sheetId="11" name="msg" state="visible" r:id="rId14"/>
+    <sheet sheetId="4" name="jobs" state="visible" r:id="rId6"/>
+    <sheet sheetId="5" name="stat" state="visible" r:id="rId7"/>
+    <sheet sheetId="6" name="tag" state="visible" r:id="rId8"/>
+    <sheet sheetId="7" name="other" state="visible" r:id="rId9"/>
+    <sheet sheetId="8" name="quest" state="visible" r:id="rId10"/>
+    <sheet sheetId="9" name="ability" state="visible" r:id="rId11"/>
+    <sheet sheetId="10" name="option" state="visible" r:id="rId12"/>
+    <sheet sheetId="11" name="msg" state="visible" r:id="rId13"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="596" uniqueCount="505">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="552" uniqueCount="470">
   <si>
     <t>key</t>
   </si>
@@ -579,178 +578,73 @@
     <t>水壺</t>
   </si>
   <si>
-    <t>wick</t>
-  </si>
-  <si>
-    <t>維克</t>
-  </si>
-  <si>
-    <t>冒險者</t>
-  </si>
-  <si>
-    <t>dummy</t>
-  </si>
-  <si>
-    <t>木樁</t>
-  </si>
-  <si>
-    <t>練習攻擊用</t>
-  </si>
-  <si>
-    <t>musk</t>
-  </si>
-  <si>
-    <t>馬斯克</t>
-  </si>
-  <si>
-    <t>寡言卻可靠的中年壯漢，鍛造技術一流，據說曾是王都兵工坊的首席</t>
-  </si>
-  <si>
-    <t>trump</t>
-  </si>
-  <si>
-    <t>川普</t>
-  </si>
-  <si>
-    <t>胖胖和氣的大叔，愛講笑話和八卦，是村裡的情報中心。</t>
-  </si>
-  <si>
-    <t>karen</t>
-  </si>
-  <si>
-    <t>凱倫</t>
-  </si>
-  <si>
-    <t>每天從村外的田地或森林帶回最新鮮的農作物，推著小車叫賣，聲音又甜又響亮～</t>
-  </si>
-  <si>
-    <t>xi</t>
-  </si>
-  <si>
-    <t>習近平</t>
-  </si>
-  <si>
-    <t>負責村裡所有牲畜的宰殺與肉品加工。據說他手起刀落，比鐵匠還俐落……</t>
-  </si>
-  <si>
-    <t>macron</t>
-  </si>
-  <si>
-    <t>馬克宏</t>
-  </si>
-  <si>
-    <t>矮個子滿臉皺紋的小老頭，總能拿出些「你不知道自己需要的東西」。</t>
-  </si>
-  <si>
-    <t>melanie</t>
-  </si>
-  <si>
-    <t>梅蘭妮</t>
-  </si>
-  <si>
-    <t>漂亮大方的女士，跟川普共同經營一家旅館</t>
+    <t>ranger</t>
+  </si>
+  <si>
+    <t>遊俠</t>
+  </si>
+  <si>
+    <t>弓箭高手、森林獵人、野外生存達人，腳步輕盈如風，氣息比幽靈還難察覺</t>
+  </si>
+  <si>
+    <t>smith</t>
+  </si>
+  <si>
+    <t>鐵匠</t>
+  </si>
+  <si>
+    <t>打造武器、防具與工具的鍛造高手。</t>
+  </si>
+  <si>
+    <t>innkeeper</t>
+  </si>
+  <si>
+    <t>旅館老闆</t>
+  </si>
+  <si>
+    <t>經營旅館與酒館，消息靈通的熱情招待。</t>
+  </si>
+  <si>
+    <t>trader</t>
+  </si>
+  <si>
+    <t>小販</t>
+  </si>
+  <si>
+    <t>村內攤商，賣日用品或冒險裝備。</t>
+  </si>
+  <si>
+    <t>butcher</t>
+  </si>
+  <si>
+    <t>屠夫</t>
+  </si>
+  <si>
+    <t>處理牲畜肉品，刀法俐落，力氣驚人。</t>
+  </si>
+  <si>
+    <t>merchant</t>
+  </si>
+  <si>
+    <t>行商</t>
+  </si>
+  <si>
+    <t>來去自如的商旅，販售異地貨品。</t>
+  </si>
+  <si>
+    <t>guard</t>
+  </si>
+  <si>
+    <t>守衛</t>
+  </si>
+  <si>
+    <t>巡邏村莊、維持治安。</t>
   </si>
   <si>
     <t>rogue</t>
   </si>
   <si>
     <t>盜賊</t>
-  </si>
-  <si>
-    <t>guard-1</t>
-  </si>
-  <si>
-    <t>守衛</t>
-  </si>
-  <si>
-    <t>駐守南門的守衛，跟搭檔輪流日夜巡邏村子</t>
-  </si>
-  <si>
-    <t>guard-2</t>
-  </si>
-  <si>
-    <t>rogue-1</t>
-  </si>
-  <si>
-    <t>rogue-2</t>
-  </si>
-  <si>
-    <t>orc</t>
-  </si>
-  <si>
-    <t>獸人</t>
-  </si>
-  <si>
-    <t>wolf</t>
-  </si>
-  <si>
-    <t>狼</t>
-  </si>
-  <si>
-    <t>horse</t>
-  </si>
-  <si>
-    <t>馬</t>
-  </si>
-  <si>
-    <t>ranger</t>
-  </si>
-  <si>
-    <t>遊俠</t>
-  </si>
-  <si>
-    <t>弓箭高手、森林獵人、野外生存達人，腳步輕盈如風，氣息比幽靈還難察覺</t>
-  </si>
-  <si>
-    <t>smith</t>
-  </si>
-  <si>
-    <t>鐵匠</t>
-  </si>
-  <si>
-    <t>打造武器、防具與工具的鍛造高手。</t>
-  </si>
-  <si>
-    <t>innkeeper</t>
-  </si>
-  <si>
-    <t>旅館老闆</t>
-  </si>
-  <si>
-    <t>經營旅館與酒館，消息靈通的熱情招待。</t>
-  </si>
-  <si>
-    <t>trader</t>
-  </si>
-  <si>
-    <t>小販</t>
-  </si>
-  <si>
-    <t>村內攤商，賣日用品或冒險裝備。</t>
-  </si>
-  <si>
-    <t>butcher</t>
-  </si>
-  <si>
-    <t>屠夫</t>
-  </si>
-  <si>
-    <t>處理牲畜肉品，刀法俐落，力氣驚人。</t>
-  </si>
-  <si>
-    <t>merchant</t>
-  </si>
-  <si>
-    <t>行商</t>
-  </si>
-  <si>
-    <t>來去自如的商旅，販售異地貨品。</t>
-  </si>
-  <si>
-    <t>guard</t>
-  </si>
-  <si>
-    <t>巡邏村莊、維持治安。</t>
   </si>
   <si>
     <t>str</t>
@@ -1639,7 +1533,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1664,9 +1558,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -2893,40 +2784,40 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>402</v>
+        <v>367</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>403</v>
+        <v>368</v>
       </c>
       <c r="D15" s="3"/>
       <c r="E15" s="3"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>404</v>
+        <v>369</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>405</v>
+        <v>370</v>
       </c>
       <c r="D16" s="3"/>
       <c r="E16" s="3"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>406</v>
+        <v>371</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>407</v>
+        <v>372</v>
       </c>
       <c r="D17" s="3"/>
       <c r="E17" s="3"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>234</v>
+        <v>196</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>408</v>
+        <v>373</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" s="3"/>
@@ -2934,10 +2825,10 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>409</v>
+        <v>374</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>410</v>
+        <v>375</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" s="3"/>
@@ -2984,421 +2875,421 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>411</v>
+        <v>376</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>412</v>
+        <v>377</v>
       </c>
       <c r="C3" s="2"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>413</v>
+        <v>378</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>414</v>
+        <v>379</v>
       </c>
       <c r="C4" s="2"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>415</v>
+        <v>380</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>416</v>
+        <v>381</v>
       </c>
       <c r="C5" s="2"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>417</v>
+        <v>382</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>418</v>
+        <v>383</v>
       </c>
       <c r="C6" s="2"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>419</v>
+        <v>384</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>420</v>
+        <v>385</v>
       </c>
       <c r="C7" s="2"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>421</v>
+        <v>386</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>422</v>
+        <v>387</v>
       </c>
       <c r="C8" s="2"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>423</v>
+        <v>388</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>424</v>
+        <v>389</v>
       </c>
       <c r="C9" s="2"/>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>425</v>
+        <v>390</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>426</v>
+        <v>391</v>
       </c>
       <c r="C10" s="2"/>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>427</v>
+        <v>392</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>428</v>
+        <v>393</v>
       </c>
       <c r="C11" s="2"/>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>429</v>
+        <v>394</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>430</v>
+        <v>395</v>
       </c>
       <c r="C12" s="2"/>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>431</v>
+        <v>396</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>432</v>
+        <v>397</v>
       </c>
       <c r="C13" s="2"/>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>433</v>
+        <v>398</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>434</v>
+        <v>399</v>
       </c>
       <c r="C14" s="2"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>435</v>
+        <v>400</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>436</v>
+        <v>401</v>
       </c>
       <c r="C15" s="2"/>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>437</v>
+        <v>402</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>438</v>
+        <v>403</v>
       </c>
       <c r="C16" s="2"/>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>439</v>
+        <v>404</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>440</v>
+        <v>405</v>
       </c>
       <c r="C17" s="2"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>441</v>
+        <v>406</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>442</v>
+        <v>407</v>
       </c>
       <c r="C18" s="2"/>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>443</v>
+        <v>408</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>444</v>
+        <v>409</v>
       </c>
       <c r="C19" s="2"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>445</v>
+        <v>410</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>446</v>
+        <v>411</v>
       </c>
       <c r="C20" s="2"/>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>447</v>
+        <v>412</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>448</v>
+        <v>413</v>
       </c>
       <c r="C21" s="2"/>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>449</v>
+        <v>414</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>450</v>
+        <v>415</v>
       </c>
       <c r="C22" s="2"/>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>451</v>
+        <v>416</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>452</v>
+        <v>417</v>
       </c>
       <c r="C23" s="2"/>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>453</v>
+        <v>418</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>454</v>
+        <v>419</v>
       </c>
       <c r="C24" s="2"/>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>455</v>
+        <v>420</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>456</v>
+        <v>421</v>
       </c>
       <c r="C25" s="2"/>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>457</v>
+        <v>422</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>458</v>
+        <v>423</v>
       </c>
       <c r="C26" s="2"/>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>459</v>
+        <v>424</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>460</v>
+        <v>425</v>
       </c>
       <c r="C27" s="2"/>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>461</v>
+        <v>426</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>462</v>
+        <v>427</v>
       </c>
       <c r="C28" s="2"/>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>463</v>
+        <v>428</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>464</v>
+        <v>429</v>
       </c>
       <c r="C29" s="2"/>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>465</v>
+        <v>430</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>466</v>
+        <v>431</v>
       </c>
       <c r="C30" s="2"/>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>467</v>
+        <v>432</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>468</v>
+        <v>433</v>
       </c>
       <c r="C31" s="2"/>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>469</v>
+        <v>434</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>470</v>
+        <v>435</v>
       </c>
       <c r="C32" s="2"/>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>471</v>
+        <v>436</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>472</v>
+        <v>437</v>
       </c>
       <c r="C33" s="2"/>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>473</v>
+        <v>438</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>474</v>
+        <v>439</v>
       </c>
       <c r="C34" s="2"/>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>475</v>
+        <v>440</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>476</v>
+        <v>441</v>
       </c>
       <c r="C35" s="2"/>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>477</v>
+        <v>442</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>478</v>
+        <v>443</v>
       </c>
       <c r="C36" s="2"/>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>479</v>
+        <v>444</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>480</v>
+        <v>445</v>
       </c>
       <c r="C37" s="2"/>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>481</v>
+        <v>446</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>482</v>
+        <v>447</v>
       </c>
       <c r="C38" s="2"/>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>483</v>
+        <v>448</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>484</v>
+        <v>449</v>
       </c>
       <c r="C39" s="2"/>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>485</v>
+        <v>450</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>486</v>
+        <v>451</v>
       </c>
       <c r="C40" s="2"/>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>487</v>
+        <v>452</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>488</v>
+        <v>453</v>
       </c>
       <c r="C41" s="2"/>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>489</v>
+        <v>454</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>490</v>
+        <v>455</v>
       </c>
       <c r="C42" s="2"/>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>491</v>
+        <v>456</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>492</v>
+        <v>457</v>
       </c>
       <c r="C43" s="2"/>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>493</v>
+        <v>458</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>494</v>
+        <v>459</v>
       </c>
       <c r="C44" s="2"/>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
-        <v>495</v>
+        <v>460</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>496</v>
+        <v>461</v>
       </c>
       <c r="C45" s="2"/>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>497</v>
+        <v>462</v>
       </c>
       <c r="B46" t="s">
-        <v>498</v>
+        <v>463</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>499</v>
+        <v>464</v>
       </c>
       <c r="B47" t="s">
-        <v>500</v>
+        <v>465</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>501</v>
+        <v>466</v>
       </c>
       <c r="B48" t="s">
-        <v>502</v>
+        <v>467</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>503</v>
+        <v>468</v>
       </c>
       <c r="B49" t="s">
-        <v>504</v>
+        <v>469</v>
       </c>
     </row>
   </sheetData>
@@ -3692,295 +3583,14 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E31"/>
-  <sheetFormatPr defaultRowHeight="16.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
-  <cols>
-    <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="14.875" style="5" customWidth="1"/>
-    <col min="3" max="3" width="42.5" style="9" customWidth="1"/>
-    <col min="4" max="4" width="19.625" style="6" customWidth="1"/>
-    <col min="5" max="5" width="11.125" style="6" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-    </row>
-    <row r="2" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B2" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>184</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>185</v>
-      </c>
-      <c r="C3" s="9" t="s">
-        <v>186</v>
-      </c>
-      <c r="D3" s="6"/>
-      <c r="E3" s="6"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
-        <v>187</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>188</v>
-      </c>
-      <c r="C4" s="9" t="s">
-        <v>189</v>
-      </c>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-    </row>
-    <row r="5" ht="33" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
-        <v>190</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>191</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>192</v>
-      </c>
-      <c r="D5" s="8"/>
-      <c r="E5" s="6"/>
-    </row>
-    <row r="6" ht="33" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
-        <v>193</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>194</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>195</v>
-      </c>
-      <c r="D6" s="8"/>
-      <c r="E6" s="6"/>
-    </row>
-    <row r="7" ht="33" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
-        <v>196</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>197</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>198</v>
-      </c>
-      <c r="D7" s="8"/>
-      <c r="E7" s="6"/>
-    </row>
-    <row r="8" ht="33" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="7" t="s">
-        <v>199</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>200</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>201</v>
-      </c>
-      <c r="D8" s="8"/>
-      <c r="E8" s="6"/>
-    </row>
-    <row r="9" ht="33" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="7" t="s">
-        <v>202</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>203</v>
-      </c>
-      <c r="C9" s="9" t="s">
-        <v>204</v>
-      </c>
-      <c r="D9" s="8"/>
-      <c r="E9" s="6"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="7" t="s">
-        <v>205</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>206</v>
-      </c>
-      <c r="C10" s="9" t="s">
-        <v>207</v>
-      </c>
-      <c r="D10" s="8"/>
-      <c r="E10" s="6"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="7"/>
-      <c r="D11" s="8"/>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="7" t="s">
-        <v>208</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>209</v>
-      </c>
-      <c r="C12" s="9"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="6"/>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="7" t="s">
-        <v>210</v>
-      </c>
-      <c r="B13" s="5" t="s">
-        <v>211</v>
-      </c>
-      <c r="C13" s="9" t="s">
-        <v>212</v>
-      </c>
-      <c r="D13" s="8"/>
-      <c r="E13" s="6"/>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="7" t="s">
-        <v>213</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>211</v>
-      </c>
-      <c r="C14" s="9" t="s">
-        <v>212</v>
-      </c>
-      <c r="D14" s="8"/>
-      <c r="E14" s="6"/>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="7" t="s">
-        <v>214</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>209</v>
-      </c>
-      <c r="C15" s="9"/>
-      <c r="D15" s="8"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="7" t="s">
-        <v>215</v>
-      </c>
-      <c r="B16" s="5" t="s">
-        <v>209</v>
-      </c>
-      <c r="C16" s="9"/>
-      <c r="D16" s="8"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="7" t="s">
-        <v>216</v>
-      </c>
-      <c r="B17" s="5" t="s">
-        <v>217</v>
-      </c>
-      <c r="C17" s="9"/>
-      <c r="D17" s="8"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="7" t="s">
-        <v>218</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>219</v>
-      </c>
-      <c r="C18" s="9"/>
-      <c r="D18" s="8"/>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>221</v>
-      </c>
-      <c r="C19" s="9"/>
-      <c r="D19" s="8"/>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="7"/>
-      <c r="D20" s="8"/>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="7"/>
-      <c r="D21" s="8"/>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="7"/>
-      <c r="D22" s="8"/>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="7"/>
-      <c r="D23" s="8"/>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="7"/>
-      <c r="D24" s="8"/>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="7"/>
-      <c r="D25" s="8"/>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="7"/>
-      <c r="D26" s="8"/>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="7"/>
-      <c r="D27" s="8"/>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="7"/>
-      <c r="D28" s="8"/>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="7"/>
-      <c r="D29" s="8"/>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="7"/>
-      <c r="D30" s="8"/>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="7"/>
-      <c r="D31" s="8"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="200" verticalDpi="200" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E31"/>
   <sheetFormatPr defaultRowHeight="15.75" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.875" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="16" style="1" customWidth="1"/>
-    <col min="2" max="2" width="14.875" style="10" customWidth="1"/>
-    <col min="3" max="3" width="42.5" style="11" customWidth="1"/>
+    <col min="2" max="2" width="14.875" style="9" customWidth="1"/>
+    <col min="3" max="3" width="42.5" style="10" customWidth="1"/>
     <col min="4" max="4" width="19.625" style="3" customWidth="1"/>
     <col min="5" max="5" width="11.125" style="3" customWidth="1"/>
     <col min="6" max="16384" width="8.875" style="1" customWidth="1"/>
@@ -3990,7 +3600,7 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="9" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="3"/>
@@ -3998,10 +3608,10 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
-      <c r="B2" s="10" t="s">
+      <c r="B2" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="C2" s="10" t="s">
         <v>3</v>
       </c>
       <c r="D2" s="3"/>
@@ -4009,13 +3619,13 @@
     </row>
     <row r="3" ht="31.5" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>222</v>
-      </c>
-      <c r="B3" s="10" t="s">
-        <v>223</v>
-      </c>
-      <c r="C3" s="11" t="s">
-        <v>224</v>
+        <v>184</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>185</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>186</v>
       </c>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
@@ -4024,86 +3634,92 @@
       <c r="A4" s="7"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="12" t="s">
-        <v>225</v>
-      </c>
-      <c r="B5" s="11" t="s">
-        <v>226</v>
-      </c>
-      <c r="C5" s="11" t="s">
-        <v>227</v>
-      </c>
-      <c r="D5" s="13"/>
+      <c r="A5" s="11" t="s">
+        <v>187</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>188</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>189</v>
+      </c>
+      <c r="D5" s="12"/>
       <c r="E5" s="3"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="12" t="s">
-        <v>228</v>
-      </c>
-      <c r="B6" s="11" t="s">
-        <v>229</v>
-      </c>
-      <c r="C6" s="11" t="s">
-        <v>230</v>
-      </c>
-      <c r="D6" s="13"/>
+      <c r="A6" s="11" t="s">
+        <v>190</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>191</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>192</v>
+      </c>
+      <c r="D6" s="12"/>
       <c r="E6" s="3"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="12" t="s">
-        <v>231</v>
-      </c>
-      <c r="B7" s="11" t="s">
-        <v>232</v>
-      </c>
-      <c r="C7" s="11" t="s">
-        <v>233</v>
-      </c>
-      <c r="D7" s="13"/>
+      <c r="A7" s="11" t="s">
+        <v>193</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>194</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="D7" s="12"/>
       <c r="E7" s="3"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="12" t="s">
-        <v>234</v>
-      </c>
-      <c r="B8" s="11" t="s">
-        <v>235</v>
-      </c>
-      <c r="C8" s="11" t="s">
-        <v>236</v>
-      </c>
-      <c r="D8" s="13"/>
+      <c r="A8" s="11" t="s">
+        <v>196</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>197</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>198</v>
+      </c>
+      <c r="D8" s="12"/>
       <c r="E8" s="3"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="12" t="s">
-        <v>237</v>
-      </c>
-      <c r="B9" s="11" t="s">
-        <v>238</v>
-      </c>
-      <c r="C9" s="11" t="s">
-        <v>239</v>
-      </c>
-      <c r="D9" s="13"/>
+      <c r="A9" s="11" t="s">
+        <v>199</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>201</v>
+      </c>
+      <c r="D9" s="12"/>
       <c r="E9" s="3"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="12" t="s">
-        <v>240</v>
-      </c>
-      <c r="B10" s="11" t="s">
-        <v>211</v>
-      </c>
-      <c r="C10" s="11" t="s">
-        <v>241</v>
-      </c>
-      <c r="D10" s="13"/>
+      <c r="A10" s="11" t="s">
+        <v>202</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>203</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>204</v>
+      </c>
+      <c r="D10" s="12"/>
       <c r="E10" s="3"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="7"/>
-      <c r="D11" s="8"/>
+      <c r="A11" s="11" t="s">
+        <v>205</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>206</v>
+      </c>
+      <c r="C11" s="10"/>
+      <c r="D11" s="12"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="7"/>
@@ -4215,338 +3831,338 @@
       <c r="E1" s="3"/>
     </row>
     <row r="2" ht="16.5" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="14"/>
-      <c r="B2" s="15" t="s">
+      <c r="A2" s="13"/>
+      <c r="B2" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="C2" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
     </row>
     <row r="3" ht="16.5" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>242</v>
-      </c>
-      <c r="B3" s="17" t="s">
-        <v>243</v>
-      </c>
-      <c r="C3" s="17" t="s">
-        <v>244</v>
+        <v>207</v>
+      </c>
+      <c r="B3" s="16" t="s">
+        <v>208</v>
+      </c>
+      <c r="C3" s="16" t="s">
+        <v>209</v>
       </c>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>245</v>
-      </c>
-      <c r="B4" s="18" t="s">
-        <v>246</v>
-      </c>
-      <c r="C4" s="18" t="s">
-        <v>247</v>
+        <v>210</v>
+      </c>
+      <c r="B4" s="17" t="s">
+        <v>211</v>
+      </c>
+      <c r="C4" s="17" t="s">
+        <v>212</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>248</v>
-      </c>
-      <c r="B5" s="18" t="s">
-        <v>249</v>
-      </c>
-      <c r="C5" s="18" t="s">
-        <v>250</v>
+        <v>213</v>
+      </c>
+      <c r="B5" s="17" t="s">
+        <v>214</v>
+      </c>
+      <c r="C5" s="17" t="s">
+        <v>215</v>
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="3"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>251</v>
-      </c>
-      <c r="B6" s="18" t="s">
-        <v>252</v>
-      </c>
-      <c r="C6" s="18" t="s">
-        <v>253</v>
+        <v>216</v>
+      </c>
+      <c r="B6" s="17" t="s">
+        <v>217</v>
+      </c>
+      <c r="C6" s="17" t="s">
+        <v>218</v>
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>254</v>
-      </c>
-      <c r="B7" s="18" t="s">
-        <v>255</v>
-      </c>
-      <c r="C7" s="18" t="s">
-        <v>256</v>
+        <v>219</v>
+      </c>
+      <c r="B7" s="17" t="s">
+        <v>220</v>
+      </c>
+      <c r="C7" s="17" t="s">
+        <v>221</v>
       </c>
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B8" s="18"/>
-      <c r="C8" s="18"/>
+      <c r="B8" s="17"/>
+      <c r="C8" s="17"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>257</v>
-      </c>
-      <c r="B9" s="18" t="s">
-        <v>258</v>
-      </c>
-      <c r="C9" s="18"/>
+        <v>222</v>
+      </c>
+      <c r="B9" s="17" t="s">
+        <v>223</v>
+      </c>
+      <c r="C9" s="17"/>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>259</v>
-      </c>
-      <c r="B10" s="18" t="s">
+        <v>224</v>
+      </c>
+      <c r="B10" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="C10" s="18" t="s">
-        <v>260</v>
+      <c r="C10" s="17" t="s">
+        <v>225</v>
       </c>
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>261</v>
-      </c>
-      <c r="B11" s="18" t="s">
+        <v>226</v>
+      </c>
+      <c r="B11" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="C11" s="18" t="s">
-        <v>262</v>
+      <c r="C11" s="17" t="s">
+        <v>227</v>
       </c>
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>263</v>
-      </c>
-      <c r="B12" s="18" t="s">
-        <v>264</v>
-      </c>
-      <c r="C12" s="18" t="s">
-        <v>265</v>
+        <v>228</v>
+      </c>
+      <c r="B12" s="17" t="s">
+        <v>229</v>
+      </c>
+      <c r="C12" s="17" t="s">
+        <v>230</v>
       </c>
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>266</v>
-      </c>
-      <c r="B13" s="18" t="s">
-        <v>267</v>
-      </c>
-      <c r="C13" s="18" t="s">
-        <v>268</v>
+        <v>231</v>
+      </c>
+      <c r="B13" s="17" t="s">
+        <v>232</v>
+      </c>
+      <c r="C13" s="17" t="s">
+        <v>233</v>
       </c>
       <c r="D13" s="3"/>
       <c r="E13" s="3"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>269</v>
-      </c>
-      <c r="B14" s="18" t="s">
-        <v>270</v>
-      </c>
-      <c r="C14" s="18" t="s">
-        <v>271</v>
+        <v>234</v>
+      </c>
+      <c r="B14" s="17" t="s">
+        <v>235</v>
+      </c>
+      <c r="C14" s="17" t="s">
+        <v>236</v>
       </c>
       <c r="D14" s="3"/>
       <c r="E14" s="3"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>272</v>
-      </c>
-      <c r="B15" s="18" t="s">
-        <v>273</v>
-      </c>
-      <c r="C15" s="18" t="s">
-        <v>274</v>
+        <v>237</v>
+      </c>
+      <c r="B15" s="17" t="s">
+        <v>238</v>
+      </c>
+      <c r="C15" s="17" t="s">
+        <v>239</v>
       </c>
       <c r="D15" s="3"/>
       <c r="E15" s="3"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>275</v>
-      </c>
-      <c r="B16" s="18" t="s">
-        <v>276</v>
-      </c>
-      <c r="C16" s="18" t="s">
-        <v>277</v>
+        <v>240</v>
+      </c>
+      <c r="B16" s="17" t="s">
+        <v>241</v>
+      </c>
+      <c r="C16" s="17" t="s">
+        <v>242</v>
       </c>
       <c r="D16" s="3"/>
       <c r="E16" s="3"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>278</v>
-      </c>
-      <c r="B17" s="18" t="s">
-        <v>279</v>
-      </c>
-      <c r="C17" s="18" t="s">
-        <v>280</v>
+        <v>243</v>
+      </c>
+      <c r="B17" s="17" t="s">
+        <v>244</v>
+      </c>
+      <c r="C17" s="17" t="s">
+        <v>245</v>
       </c>
       <c r="D17" s="3"/>
       <c r="E17" s="3"/>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B18" s="18"/>
-      <c r="C18" s="18"/>
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>281</v>
-      </c>
-      <c r="B19" s="18" t="s">
-        <v>282</v>
-      </c>
-      <c r="C19" s="18"/>
+        <v>246</v>
+      </c>
+      <c r="B19" s="17" t="s">
+        <v>247</v>
+      </c>
+      <c r="C19" s="17"/>
       <c r="D19" s="3"/>
       <c r="E19" s="3"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>283</v>
-      </c>
-      <c r="B20" s="18" t="s">
-        <v>284</v>
-      </c>
-      <c r="C20" s="18" t="s">
-        <v>285</v>
+        <v>248</v>
+      </c>
+      <c r="B20" s="17" t="s">
+        <v>249</v>
+      </c>
+      <c r="C20" s="17" t="s">
+        <v>250</v>
       </c>
       <c r="D20" s="3"/>
       <c r="E20" s="3"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>286</v>
-      </c>
-      <c r="B21" s="18" t="s">
-        <v>287</v>
-      </c>
-      <c r="C21" s="18" t="s">
-        <v>288</v>
+        <v>251</v>
+      </c>
+      <c r="B21" s="17" t="s">
+        <v>252</v>
+      </c>
+      <c r="C21" s="17" t="s">
+        <v>253</v>
       </c>
       <c r="D21" s="3"/>
       <c r="E21" s="3"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>289</v>
-      </c>
-      <c r="B22" s="18" t="s">
-        <v>290</v>
-      </c>
-      <c r="C22" s="18" t="s">
-        <v>291</v>
+        <v>254</v>
+      </c>
+      <c r="B22" s="17" t="s">
+        <v>255</v>
+      </c>
+      <c r="C22" s="17" t="s">
+        <v>256</v>
       </c>
       <c r="D22" s="3"/>
       <c r="E22" s="3"/>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>292</v>
-      </c>
-      <c r="B23" s="18" t="s">
-        <v>293</v>
-      </c>
-      <c r="C23" s="18" t="s">
-        <v>294</v>
+        <v>257</v>
+      </c>
+      <c r="B23" s="17" t="s">
+        <v>258</v>
+      </c>
+      <c r="C23" s="17" t="s">
+        <v>259</v>
       </c>
       <c r="D23" s="3"/>
       <c r="E23" s="3"/>
     </row>
     <row r="24" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B24" s="18"/>
-      <c r="C24" s="18"/>
+      <c r="B24" s="17"/>
+      <c r="C24" s="17"/>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>295</v>
-      </c>
-      <c r="B25" s="18" t="s">
-        <v>296</v>
-      </c>
-      <c r="C25" s="18"/>
+        <v>260</v>
+      </c>
+      <c r="B25" s="17" t="s">
+        <v>261</v>
+      </c>
+      <c r="C25" s="17"/>
       <c r="D25" s="3"/>
       <c r="E25" s="3"/>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>297</v>
-      </c>
-      <c r="B26" s="18" t="s">
-        <v>298</v>
-      </c>
-      <c r="C26" s="18"/>
+        <v>262</v>
+      </c>
+      <c r="B26" s="17" t="s">
+        <v>263</v>
+      </c>
+      <c r="C26" s="17"/>
       <c r="D26" s="3"/>
       <c r="E26" s="3"/>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>299</v>
-      </c>
-      <c r="B27" s="18" t="s">
-        <v>300</v>
-      </c>
-      <c r="C27" s="18"/>
+        <v>264</v>
+      </c>
+      <c r="B27" s="17" t="s">
+        <v>265</v>
+      </c>
+      <c r="C27" s="17"/>
       <c r="D27" s="3"/>
       <c r="E27" s="3"/>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="B28" s="18" t="s">
-        <v>302</v>
-      </c>
-      <c r="C28" s="18"/>
+        <v>266</v>
+      </c>
+      <c r="B28" s="17" t="s">
+        <v>267</v>
+      </c>
+      <c r="C28" s="17"/>
       <c r="D28" s="3"/>
       <c r="E28" s="3"/>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>303</v>
-      </c>
-      <c r="B29" s="18" t="s">
-        <v>304</v>
-      </c>
-      <c r="C29" s="18"/>
+        <v>268</v>
+      </c>
+      <c r="B29" s="17" t="s">
+        <v>269</v>
+      </c>
+      <c r="C29" s="17"/>
       <c r="D29" s="3"/>
       <c r="E29" s="3"/>
     </row>
     <row r="30" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B30" s="18"/>
-      <c r="C30" s="18"/>
+      <c r="B30" s="17"/>
+      <c r="C30" s="17"/>
     </row>
     <row r="31" ht="31.5" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>305</v>
-      </c>
-      <c r="B31" s="18" t="s">
+        <v>270</v>
+      </c>
+      <c r="B31" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="C31" s="19" t="s">
+      <c r="C31" s="18" t="s">
         <v>49</v>
       </c>
       <c r="D31" s="3"/>
@@ -4554,168 +4170,168 @@
     </row>
     <row r="32" ht="31.5" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>306</v>
-      </c>
-      <c r="B32" s="18" t="s">
-        <v>307</v>
-      </c>
-      <c r="C32" s="19" t="s">
-        <v>308</v>
+        <v>271</v>
+      </c>
+      <c r="B32" s="17" t="s">
+        <v>272</v>
+      </c>
+      <c r="C32" s="18" t="s">
+        <v>273</v>
       </c>
       <c r="D32" s="3"/>
       <c r="E32" s="3"/>
     </row>
     <row r="33" ht="31.5" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>309</v>
-      </c>
-      <c r="B33" s="18" t="s">
-        <v>310</v>
-      </c>
-      <c r="C33" s="19" t="s">
-        <v>311</v>
+        <v>274</v>
+      </c>
+      <c r="B33" s="17" t="s">
+        <v>275</v>
+      </c>
+      <c r="C33" s="18" t="s">
+        <v>276</v>
       </c>
       <c r="D33" s="3"/>
       <c r="E33" s="3"/>
     </row>
     <row r="34" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B34" s="18"/>
-      <c r="C34" s="18"/>
+      <c r="B34" s="17"/>
+      <c r="C34" s="17"/>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>312</v>
-      </c>
-      <c r="B35" s="18" t="s">
-        <v>313</v>
-      </c>
-      <c r="C35" s="19" t="s">
-        <v>314</v>
+        <v>277</v>
+      </c>
+      <c r="B35" s="17" t="s">
+        <v>278</v>
+      </c>
+      <c r="C35" s="18" t="s">
+        <v>279</v>
       </c>
       <c r="D35" s="3"/>
       <c r="E35" s="3"/>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>315</v>
-      </c>
-      <c r="B36" s="18" t="s">
-        <v>316</v>
-      </c>
-      <c r="C36" s="19" t="s">
-        <v>317</v>
+        <v>280</v>
+      </c>
+      <c r="B36" s="17" t="s">
+        <v>281</v>
+      </c>
+      <c r="C36" s="18" t="s">
+        <v>282</v>
       </c>
       <c r="D36" s="3"/>
       <c r="E36" s="3"/>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>318</v>
-      </c>
-      <c r="B37" s="18" t="s">
-        <v>319</v>
-      </c>
-      <c r="C37" s="19" t="s">
-        <v>320</v>
+        <v>283</v>
+      </c>
+      <c r="B37" s="17" t="s">
+        <v>284</v>
+      </c>
+      <c r="C37" s="18" t="s">
+        <v>285</v>
       </c>
       <c r="D37" s="3"/>
       <c r="E37" s="3"/>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>321</v>
-      </c>
-      <c r="B39" s="18" t="s">
-        <v>313</v>
-      </c>
-      <c r="C39" s="19" t="s">
-        <v>322</v>
+        <v>286</v>
+      </c>
+      <c r="B39" s="17" t="s">
+        <v>278</v>
+      </c>
+      <c r="C39" s="18" t="s">
+        <v>287</v>
       </c>
       <c r="D39" s="3"/>
       <c r="E39" s="3"/>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>323</v>
-      </c>
-      <c r="B40" s="18" t="s">
-        <v>316</v>
-      </c>
-      <c r="C40" s="19" t="s">
-        <v>324</v>
+        <v>288</v>
+      </c>
+      <c r="B40" s="17" t="s">
+        <v>281</v>
+      </c>
+      <c r="C40" s="18" t="s">
+        <v>289</v>
       </c>
       <c r="D40" s="3"/>
       <c r="E40" s="3"/>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>325</v>
+        <v>290</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>319</v>
+        <v>284</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>326</v>
+        <v>291</v>
       </c>
       <c r="D41" s="3"/>
       <c r="E41" s="3"/>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>327</v>
+        <v>292</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>328</v>
+        <v>293</v>
       </c>
       <c r="D43" s="3"/>
       <c r="E43" s="3"/>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>329</v>
+        <v>294</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>330</v>
+        <v>295</v>
       </c>
       <c r="D44" s="3"/>
       <c r="E44" s="3"/>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
-        <v>331</v>
+        <v>296</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>267</v>
+        <v>232</v>
       </c>
       <c r="D45" s="3"/>
       <c r="E45" s="3"/>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
-        <v>332</v>
+        <v>297</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>333</v>
+        <v>298</v>
       </c>
       <c r="D46" s="3"/>
       <c r="E46" s="3"/>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
-        <v>334</v>
+        <v>299</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>335</v>
+        <v>300</v>
       </c>
       <c r="D48" s="3"/>
       <c r="E48" s="3"/>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
-        <v>336</v>
+        <v>301</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>337</v>
+        <v>302</v>
       </c>
       <c r="C49" s="4"/>
       <c r="D49" s="3"/>
@@ -4723,33 +4339,33 @@
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
-        <v>338</v>
+        <v>303</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>339</v>
+        <v>304</v>
       </c>
       <c r="D51" s="3"/>
       <c r="E51" s="3"/>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
-        <v>340</v>
+        <v>305</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>341</v>
+        <v>306</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>342</v>
+        <v>307</v>
       </c>
       <c r="D52" s="3"/>
       <c r="E52" s="3"/>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
-        <v>343</v>
+        <v>308</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>344</v>
+        <v>309</v>
       </c>
       <c r="C53" s="4"/>
       <c r="D53" s="3"/>
@@ -4757,40 +4373,40 @@
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
-        <v>345</v>
+        <v>310</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>346</v>
+        <v>311</v>
       </c>
       <c r="D54" s="3"/>
       <c r="E54" s="3"/>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
-        <v>347</v>
+        <v>312</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>348</v>
+        <v>313</v>
       </c>
       <c r="D55" s="3"/>
       <c r="E55" s="3"/>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
-        <v>349</v>
+        <v>314</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>350</v>
+        <v>315</v>
       </c>
       <c r="D56" s="3"/>
       <c r="E56" s="3"/>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
-        <v>351</v>
+        <v>316</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>352</v>
+        <v>317</v>
       </c>
       <c r="D57" s="3"/>
       <c r="E57" s="3"/>
@@ -4822,39 +4438,39 @@
       <c r="E1" s="3"/>
     </row>
     <row r="2" ht="17.25" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="14"/>
-      <c r="B2" s="15" t="s">
+      <c r="A2" s="13"/>
+      <c r="B2" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="C2" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
     </row>
     <row r="3" ht="17.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>353</v>
+        <v>318</v>
       </c>
       <c r="B4" t="s">
-        <v>354</v>
+        <v>319</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>355</v>
+        <v>320</v>
       </c>
       <c r="B5" t="s">
-        <v>356</v>
+        <v>321</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>357</v>
+        <v>322</v>
       </c>
       <c r="B6" t="s">
-        <v>358</v>
+        <v>323</v>
       </c>
     </row>
   </sheetData>
@@ -4886,33 +4502,33 @@
       <c r="E1" s="3"/>
     </row>
     <row r="2" ht="16.5" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="14"/>
-      <c r="B2" s="15" t="s">
+      <c r="A2" s="13"/>
+      <c r="B2" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="C2" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
     </row>
     <row r="3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>359</v>
+        <v>324</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>360</v>
+        <v>325</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>361</v>
+        <v>326</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>362</v>
+        <v>327</v>
       </c>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
@@ -4929,33 +4545,33 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>363</v>
+        <v>328</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>346</v>
+        <v>311</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>364</v>
+        <v>329</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>365</v>
+        <v>330</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>366</v>
+        <v>331</v>
       </c>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>367</v>
+        <v>332</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>368</v>
+        <v>333</v>
       </c>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
@@ -4970,10 +4586,10 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>369</v>
+        <v>334</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>370</v>
+        <v>335</v>
       </c>
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
@@ -4981,10 +4597,10 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>371</v>
+        <v>336</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>372</v>
+        <v>337</v>
       </c>
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
@@ -4992,10 +4608,10 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>373</v>
+        <v>338</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>374</v>
+        <v>339</v>
       </c>
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
@@ -5032,63 +4648,63 @@
       <c r="E1" s="3"/>
     </row>
     <row r="2" ht="16.5" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="14"/>
-      <c r="B2" s="15" t="s">
+      <c r="A2" s="13"/>
+      <c r="B2" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="C2" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
     </row>
     <row r="3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>375</v>
+        <v>340</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>376</v>
+        <v>341</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>377</v>
+        <v>342</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>378</v>
+        <v>343</v>
       </c>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>379</v>
+        <v>344</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>380</v>
+        <v>345</v>
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>381</v>
+        <v>346</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>382</v>
+        <v>347</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>383</v>
+        <v>348</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>384</v>
+        <v>349</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -5130,74 +4746,74 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>385</v>
+        <v>350</v>
       </c>
       <c r="B3" t="s">
-        <v>386</v>
+        <v>351</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>387</v>
+        <v>352</v>
       </c>
       <c r="B4" t="s">
-        <v>388</v>
+        <v>353</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>389</v>
+        <v>354</v>
       </c>
       <c r="B5" t="s">
-        <v>390</v>
+        <v>355</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>391</v>
+        <v>356</v>
       </c>
       <c r="B6" t="s">
-        <v>392</v>
+        <v>357</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>393</v>
+        <v>358</v>
       </c>
       <c r="B7" t="s">
-        <v>394</v>
+        <v>359</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>395</v>
+        <v>360</v>
       </c>
       <c r="B8" t="s">
-        <v>396</v>
+        <v>361</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>397</v>
+        <v>362</v>
       </c>
       <c r="B9" t="s">
-        <v>398</v>
+        <v>363</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>399</v>
+        <v>364</v>
       </c>
       <c r="B10" t="s">
-        <v>358</v>
+        <v>323</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>400</v>
+        <v>365</v>
       </c>
       <c r="B12" t="s">
-        <v>401</v>
+        <v>366</v>
       </c>
     </row>
   </sheetData>

</xml_diff>